<commit_message>
chore(output): regenerer les artefacts xlsx sans remplissage colore
</commit_message>
<xml_diff>
--- a/test_output/2017/Communes/educ.xlsx
+++ b/test_output/2017/Communes/educ.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="com" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="com" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,18 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -57,7 +51,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>